<commit_message>
feat(security): close exposed surfaces and document system architecture
</commit_message>
<xml_diff>
--- a/antibiotic_dose.xlsx
+++ b/antibiotic_dose.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WEB DESIGN IT\IDEA\MedMinders\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C689399-7534-4754-A7F2-6B5CFE6ED528}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995C7BEF-16BD-4A29-9FEA-8F216F45F70F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="তুমি আমাকে এখন।পর্যন্ত যতগুলো অ" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="153">
   <si>
     <t>জেনেরিক নাম</t>
   </si>
@@ -722,69 +722,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="42">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -824,7 +794,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
@@ -851,7 +821,7 @@
     <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1204,31 +1174,31 @@
   <dimension ref="A1:H47"/>
   <sheetFormatPr defaultColWidth="37" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="5" max="5" width="117.77734375" style="35" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="51.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="68.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="117.81640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="51.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="68.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1" thickBot="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="38" t="s">
+      <c r="G1" s="28" t="s">
         <v>116</v>
       </c>
     </row>
@@ -1245,173 +1215,173 @@
       <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="51" t="s">
+      <c r="E2" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="F2" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="G2" s="37" t="s">
+      <c r="G2" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="H2" s="3"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="25"/>
+      <c r="E3" s="15"/>
     </row>
     <row r="4" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="15"/>
     </row>
     <row r="5" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="37" t="s">
+      <c r="F5" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="G5" s="37" t="s">
+      <c r="G5" s="27" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="4" t="s">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="26"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="4" t="s">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="26"/>
+      <c r="E7" s="16"/>
     </row>
     <row r="8" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="G8" s="37" t="s">
+      <c r="G8" s="27" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="6" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="27"/>
+      <c r="E9" s="17"/>
     </row>
     <row r="10" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="6" t="s">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="27"/>
+      <c r="E10" s="17"/>
     </row>
     <row r="11" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="37" t="s">
+      <c r="F11" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="G11" s="37" t="s">
+      <c r="G11" s="27" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="8" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="28"/>
+      <c r="E12" s="18"/>
     </row>
     <row r="13" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="8" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="28"/>
+      <c r="E13" s="18"/>
     </row>
     <row r="14" spans="1:8" ht="22.5" customHeight="1">
       <c r="A14" s="1" t="s">
@@ -1426,154 +1396,154 @@
       <c r="D14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="F14" s="27" t="s">
         <v>125</v>
       </c>
-      <c r="G14" s="37" t="s">
+      <c r="G14" s="27" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
       <c r="C15" s="1" t="s">
         <v>60</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="25"/>
+      <c r="E15" s="15"/>
     </row>
     <row r="16" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
       <c r="C16" s="1" t="s">
         <v>65</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="25"/>
+      <c r="E16" s="15"/>
     </row>
     <row r="17" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E17" s="43" t="s">
+      <c r="E17" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="F17" s="37" t="s">
+      <c r="F17" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="G17" s="37" t="s">
+      <c r="G17" s="27" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E18" s="44" t="s">
+      <c r="E18" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="37" t="s">
+      <c r="F18" s="27" t="s">
         <v>129</v>
       </c>
-      <c r="G18" s="37" t="s">
+      <c r="G18" s="27" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="12" t="s">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="29"/>
-      <c r="F19" s="46"/>
-      <c r="G19" s="46"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
     </row>
     <row r="20" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="12" t="s">
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E20" s="29"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
     </row>
     <row r="21" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="45" t="s">
+      <c r="E21" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="37" t="s">
+      <c r="F21" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="G21" s="37" t="s">
+      <c r="G21" s="27" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="14" t="s">
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E22" s="30"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A23" s="15"/>
-      <c r="B23" s="15"/>
-      <c r="C23" s="14" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="D23" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E23" s="30"/>
+      <c r="E23" s="20"/>
     </row>
     <row r="24" spans="1:7" ht="22.5" customHeight="1">
       <c r="A24" s="1" t="s">
@@ -1588,206 +1558,206 @@
       <c r="D24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E24" s="39" t="s">
+      <c r="E24" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="F24" s="37" t="s">
+      <c r="F24" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="G24" s="37" t="s">
+      <c r="G24" s="27" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
         <v>87</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E25" s="47"/>
+      <c r="E25" s="37"/>
     </row>
     <row r="26" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
         <v>89</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E26" s="25"/>
+      <c r="E26" s="15"/>
     </row>
     <row r="27" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E27" s="25"/>
+      <c r="E27" s="15"/>
     </row>
     <row r="28" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E28" s="48" t="s">
+      <c r="E28" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="F28" s="37" t="s">
+      <c r="F28" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="G28" s="37" t="s">
+      <c r="G28" s="27" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A29" s="17"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="16" t="s">
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="E29" s="31"/>
+      <c r="E29" s="21"/>
     </row>
     <row r="30" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="E30" s="49" t="s">
+      <c r="E30" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="F30" s="37" t="s">
+      <c r="F30" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="G30" s="37" t="s">
+      <c r="G30" s="27" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="18" t="s">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="E31" s="32"/>
+      <c r="E31" s="22"/>
     </row>
     <row r="32" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A32" s="19"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="18" t="s">
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="E32" s="32"/>
+      <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C33" s="20" t="s">
+      <c r="C33" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E33" s="50" t="s">
+      <c r="E33" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="F33" s="37" t="s">
+      <c r="F33" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="G33" s="37" t="s">
+      <c r="G33" s="27" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A34" s="21"/>
-      <c r="B34" s="21"/>
-      <c r="C34" s="20" t="s">
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="D34" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E34" s="33"/>
+      <c r="E34" s="23"/>
     </row>
     <row r="35" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A35" s="21"/>
-      <c r="B35" s="21"/>
-      <c r="C35" s="20" t="s">
+      <c r="A35" s="11"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="D35" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E35" s="33"/>
+      <c r="E35" s="23"/>
     </row>
     <row r="36" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A36" s="8" t="s">
+      <c r="A36" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D36" s="8" t="s">
+      <c r="D36" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E36" s="42" t="s">
+      <c r="E36" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="F36" s="37" t="s">
+      <c r="F36" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="G36" s="37" t="s">
+      <c r="G36" s="27" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="8" t="s">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E37" s="28"/>
+      <c r="E37" s="18"/>
     </row>
     <row r="38" spans="1:7" ht="22.5" customHeight="1">
       <c r="A38" s="1" t="s">
@@ -1802,162 +1772,162 @@
       <c r="D38" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E38" s="39" t="s">
+      <c r="E38" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="F38" s="37" t="s">
+      <c r="F38" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="G38" s="37" t="s">
+      <c r="G38" s="27" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
       <c r="C39" s="1" t="s">
         <v>106</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E39" s="25"/>
+      <c r="E39" s="15"/>
     </row>
     <row r="40" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="D40" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E40" s="40" t="s">
+      <c r="E40" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="F40" s="37" t="s">
+      <c r="F40" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="G40" s="37" t="s">
+      <c r="G40" s="27" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
-      <c r="C41" s="4" t="s">
+      <c r="A41" s="3"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E41" s="26"/>
+      <c r="E41" s="16"/>
     </row>
     <row r="42" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A42" s="10" t="s">
+      <c r="A42" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B42" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E42" s="43" t="s">
+      <c r="E42" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="F42" s="37" t="s">
+      <c r="F42" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="G42" s="37" t="s">
+      <c r="G42" s="27" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="10" t="s">
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E43" s="34"/>
+      <c r="E43" s="24"/>
     </row>
     <row r="44" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D44" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="E44" s="41" t="s">
+      <c r="E44" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="F44" s="37" t="s">
+      <c r="F44" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="G44" s="37" t="s">
+      <c r="G44" s="27" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="6" t="s">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E45" s="27"/>
+      <c r="E45" s="17"/>
     </row>
     <row r="46" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A46" s="16" t="s">
+      <c r="A46" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="B46" s="16" t="s">
+      <c r="B46" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="D46" s="16" t="s">
+      <c r="D46" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E46" s="48" t="s">
+      <c r="E46" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="F46" s="37" t="s">
+      <c r="F46" s="27" t="s">
         <v>151</v>
       </c>
-      <c r="G46" s="37" t="s">
+      <c r="G46" s="27" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A47" s="17"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="16" t="s">
+      <c r="A47" s="9"/>
+      <c r="B47" s="9"/>
+      <c r="C47" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="D47" s="16" t="s">
+      <c r="D47" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E47" s="31"/>
+      <c r="E47" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>